<commit_message>
Prepare v1.0.3 submission reproducibility update
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Table_4.xlsx
+++ b/supplementary_tables/Supplementary_Table_4.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra4ff3e41d2654e4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronology" sheetId="2" r:id="Rbb3338b544204b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R00c345e3810e40cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronology" sheetId="2" r:id="R76728c1a3e6049ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -544,7 +544,7 @@
         <x:v>scope</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="80" hidden="0" customHeight="1">
       <x:c r="A2" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -552,13 +552,13 @@
         <x:v>Development of the main analysis plan</x:v>
       </x:c>
       <x:c r="C2" s="29" t="str">
-        <x:v>Before final episode construction and reported model fitting</x:v>
+        <x:v>Local analysis-plan record dated 3 September 2026</x:v>
       </x:c>
       <x:c r="D2" s="16" t="str">
         <x:v>Cohort, event, outcome, contamination, model and validation rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="80" hidden="0" customHeight="1">
       <x:c r="A3" s="12" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -566,13 +566,13 @@
         <x:v>Specification of item-level and alternative-representation analyses</x:v>
       </x:c>
       <x:c r="C3" s="30" t="str">
-        <x:v>Before those analyses were run</x:v>
+        <x:v>Separate local plan dated 3 September 2026</x:v>
       </x:c>
       <x:c r="D3" s="17" t="str">
         <x:v>Item mapping, scale halves and alternative history representations</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="92" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -586,7 +586,7 @@
         <x:v>Recurrent caregiving and multiple prior acute-response questions; https://osf.io/zgeb3/</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="160" hidden="0" customHeight="1">
       <x:c r="A5" s="14" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -594,10 +594,10 @@
         <x:v>Pre-estimation implementation note</x:v>
       </x:c>
       <x:c r="C5" s="31" t="str">
-        <x:v>Before registered model fitting</x:v>
+        <x:v>4 September 2026, 04:27:22 UTC; sealed at 04:28:21 UTC, before the recorded extension fit start at 04:36:30 UTC</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
-        <x:v>Training-fold standardization, temporal cutoff and Gaussian predictive density</x:v>
+        <x:v>Separate technical operationalization of training-fold standardization, temporal cutoff and Gaussian predictive density; not part of the original registration</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>